<commit_message>
Migrate departments-and-units; repackage JCR (6 pages)
- Add source HTML for /lsa/academics/departments-and-units (academics-directory
  template, departms mode): intro images/text + A-Z list of ~130 department/unit
  links. Static default content (unlike majors-minors' AJAX widget), converts cleanly.
- generate-jcr.mjs: add departments-and-units to PAGES.
- Rebuild dist/lsa-eds-ue-content.zip → now 6/6 pages, all well-formed XML:
  index, lsa/prospective-students, lsa/academics/majors-minors (intro only),
  lsa/academics/departments-and-units, en/nav, en/footer.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-academics-directory.report.xlsx
+++ b/tools/importer/reports/import-academics-directory.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="63">
   <si>
     <t>_reportFile</t>
   </si>
@@ -106,7 +106,7 @@
     <t>index</t>
   </si>
   <si>
-    <t>2026-08-13T18:37:56.910Z</t>
+    <t>2026-08-13T19:09:49.009Z</t>
   </si>
   <si>
     <t>http://localhost:8082/</t>
@@ -148,7 +148,7 @@
     <t>audience-landing</t>
   </si>
   <si>
-    <t>2026-08-13T18:37:51.030Z</t>
+    <t>2026-08-13T19:09:54.180Z</t>
   </si>
   <si>
     <t>Prospective Students | U-M LSA U-M College of LSA</t>
@@ -157,16 +157,53 @@
     <t>http://localhost:8082/lsa/prospective-students.html</t>
   </si>
   <si>
+    <t>lsa/academics/departments-and-units.html.report.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.goto: net::ERR_CONNECTION_REFUSED at http://localhost:8082/lsa/academics/departments-and-units.html
+Call log:
+  - navigating to "http://localhost:8082/lsa/academics/departments-and-units.html", waiting until "domcontentloaded"
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">page.goto: net::ERR_CONNECTION_REFUSED at http://localhost:8082/lsa/academics/departments-and-units.html
+Call log:
+  - navigating to "http://localhost:8082/lsa/academics/departments-and-units.html", waiting until "domcontentloaded"
+    at processUrl (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:469:18)
+    at async main (/home/node/.excat-marketplaces/excat-marketplace/excat/skills/excat-content-import/scripts/run-bulk-import.js:696:22)</t>
+  </si>
+  <si>
+    <t>lsa/academics/departments-and-units.html</t>
+  </si>
+  <si>
+    <t>2026-08-14T14:25:12.612Z</t>
+  </si>
+  <si>
+    <t>http://localhost:8082/lsa/academics/departments-and-units.html</t>
+  </si>
+  <si>
+    <t>lsa/academics/departments-and-units.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>lsa/academics/departments-and-units</t>
+  </si>
+  <si>
+    <t>academics-listing</t>
+  </si>
+  <si>
+    <t>2026-08-14T14:25:35.515Z</t>
+  </si>
+  <si>
+    <t>Departments and Units | U-M LSA U-M College of LSA</t>
+  </si>
+  <si>
     <t>lsa/academics/majors-minors.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>lsa/academics/majors-minors</t>
-  </si>
-  <si>
-    <t>academics-listing</t>
   </si>
   <si>
     <t>2026-08-13T18:48:55.438Z</t>
@@ -564,13 +601,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K8"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="41" customWidth="1"/>
-    <col min="2" max="4" width="50" customWidth="1"/>
+    <col min="1" max="4" width="50" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
-    <col min="6" max="6" width="29" customWidth="1"/>
+    <col min="6" max="6" width="42" customWidth="1"/>
     <col min="8" max="8" width="19" customWidth="1"/>
     <col min="9" max="9" width="26" customWidth="1"/>
     <col min="10" max="11" width="50" customWidth="1"/>
@@ -826,34 +862,104 @@
         <v>46</v>
       </c>
       <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" t="s">
         <v>47</v>
       </c>
-      <c r="C8" t="s">
-        <v>12</v>
-      </c>
       <c r="D8" t="s">
-        <v>12</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
         <v>12</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G8" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="I8" t="s">
         <v>50</v>
       </c>
       <c r="J8" t="s">
+        <v>12</v>
+      </c>
+      <c r="K8" t="s">
         <v>51</v>
       </c>
-      <c r="K8" t="s">
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>52</v>
+      </c>
+      <c r="B9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C9" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="s">
+        <v>54</v>
+      </c>
+      <c r="G9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" t="s">
+        <v>56</v>
+      </c>
+      <c r="J9" t="s">
+        <v>57</v>
+      </c>
+      <c r="K9" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>59</v>
+      </c>
+      <c r="G10" t="s">
+        <v>22</v>
+      </c>
+      <c r="H10" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" t="s">
+        <v>60</v>
+      </c>
+      <c r="J10" t="s">
+        <v>61</v>
+      </c>
+      <c r="K10" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>